<commit_message>
Make name generation robust
</commit_message>
<xml_diff>
--- a/docs/_attachments/some_file_probands_only.xlsx
+++ b/docs/_attachments/some_file_probands_only.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\bodyloop\bodyloop-dashboards\docs\_attachments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127BA77E-FC3E-4C66-B81D-08507EE9ABC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FBCA78E-69D8-4BB9-89F1-06A4CF16A8E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="5892" windowWidth="30936" windowHeight="19416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>ID</t>
   </si>
@@ -61,6 +61,24 @@
   </si>
   <si>
     <t>e39f63d1-e3a3-48d9-9f15-a40f245df619</t>
+  </si>
+  <si>
+    <t>048eb97d-d466-44c1-be55-a73e9a66369e</t>
+  </si>
+  <si>
+    <t>A B C</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>A B-C</t>
+  </si>
+  <si>
+    <t>5524dfb0-50fd-40f0-9f82-614fb5a41e70</t>
+  </si>
+  <si>
+    <t>a48681b4-3cab-4cec-80ba-b930605c0bd3</t>
   </si>
 </sst>
 </file>
@@ -379,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
@@ -434,6 +452,39 @@
         <v>40544</v>
       </c>
     </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="1">
+        <v>40909</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="1">
+        <v>41275</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1">
+        <v>41640</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>